<commit_message>
chore(data-release): publish site data 2026-08-11 10:17:49 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -3081,7 +3081,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK33" t="inlineStr">
@@ -8065,7 +8065,7 @@
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
@@ -11149,7 +11149,7 @@
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK69" t="inlineStr">
@@ -11388,7 +11388,7 @@
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK70" t="inlineStr">
@@ -14911,7 +14911,7 @@
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK93" t="inlineStr">
@@ -15307,7 +15307,7 @@
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK95" t="inlineStr">
@@ -16004,7 +16004,7 @@
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK99" t="inlineStr">
@@ -16243,7 +16243,7 @@
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.7</t>
+          <t>globalid-disease-ontology:2026.08.8</t>
         </is>
       </c>
       <c r="AK100" t="inlineStr">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-11 11:15:35 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -16858,16 +16858,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>318</v>
+        <v>375</v>
       </c>
       <c r="O104" t="n">
-        <v>318</v>
+        <v>375</v>
       </c>
       <c r="Q104" t="n">
         <v>0</v>
       </c>
       <c r="R104" t="n">
-        <v>0.1489024300040756</v>
+        <v>0.1755924882123533</v>
       </c>
       <c r="S104" t="inlineStr">
         <is>
@@ -17450,16 +17450,16 @@
         </is>
       </c>
       <c r="N108" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="O108" t="n">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="Q108" t="n">
         <v>0</v>
       </c>
       <c r="R108" t="n">
-        <v>0.02060285195024946</v>
+        <v>0.0332455111015389</v>
       </c>
       <c r="S108" t="inlineStr">
         <is>
@@ -18438,16 +18438,16 @@
         </is>
       </c>
       <c r="N114" t="n">
-        <v>22</v>
+        <v>219</v>
       </c>
       <c r="O114" t="n">
-        <v>22</v>
+        <v>219</v>
       </c>
       <c r="Q114" t="n">
         <v>0</v>
       </c>
       <c r="R114" t="n">
-        <v>0.01030142597512473</v>
+        <v>0.1025460131160144</v>
       </c>
       <c r="S114" t="inlineStr">
         <is>
@@ -18586,16 +18586,16 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O115" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q115" t="n">
         <v>0</v>
       </c>
       <c r="R115" t="n">
-        <v>0.0009364932704658844</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S115" t="inlineStr">
         <is>
@@ -19178,16 +19178,16 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="O119" t="n">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="Q119" t="n">
         <v>0</v>
       </c>
       <c r="R119" t="n">
-        <v>0.001872986540931769</v>
+        <v>0.02294408512641417</v>
       </c>
       <c r="S119" t="inlineStr">
         <is>
@@ -20242,6 +20242,154 @@
         </is>
       </c>
       <c r="BC125" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>D120</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>破伤风</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N126" t="n">
+        <v>1</v>
+      </c>
+      <c r="O126" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>0</v>
+      </c>
+      <c r="R126" t="n">
+        <v>0.0004682466352329422</v>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO126" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP126" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR126" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS126" t="inlineStr"/>
+      <c r="AT126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU126" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV126" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW126" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX126" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY126" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ126" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA126" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB126" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC126" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -20363,7 +20511,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10">
@@ -20373,7 +20521,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11">
@@ -20425,7 +20573,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1012734</v>
+        <v>1013060</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-12 11:15:51 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -3081,7 +3081,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK33" t="inlineStr">
@@ -8065,7 +8065,7 @@
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
@@ -11149,7 +11149,7 @@
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK69" t="inlineStr">
@@ -11388,7 +11388,7 @@
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK70" t="inlineStr">
@@ -14911,7 +14911,7 @@
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK93" t="inlineStr">
@@ -15307,7 +15307,7 @@
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK95" t="inlineStr">
@@ -16004,7 +16004,7 @@
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK99" t="inlineStr">
@@ -16243,7 +16243,7 @@
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.8</t>
+          <t>globalid-disease-ontology:2026.08.10</t>
         </is>
       </c>
       <c r="AK100" t="inlineStr">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-14 02:00:15 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -2837,9 +2837,6 @@
       <c r="O16" t="n">
         <v>0</v>
       </c>
-      <c r="Q16" t="n">
-        <v>0</v>
-      </c>
       <c r="R16" t="n">
         <v>0</v>
       </c>
@@ -5329,9 +5326,6 @@
       <c r="O32" t="n">
         <v>14</v>
       </c>
-      <c r="Q32" t="n">
-        <v>0</v>
-      </c>
       <c r="R32" t="n">
         <v>0.006555452893261191</v>
       </c>
@@ -7821,9 +7815,6 @@
       <c r="O48" t="n">
         <v>50</v>
       </c>
-      <c r="Q48" t="n">
-        <v>0</v>
-      </c>
       <c r="R48" t="n">
         <v>0.02341233176164711</v>
       </c>
@@ -8537,9 +8528,6 @@
       <c r="O52" t="n">
         <v>1</v>
       </c>
-      <c r="Q52" t="n">
-        <v>0</v>
-      </c>
       <c r="R52" t="n">
         <v>0.0004682466352329422</v>
       </c>
@@ -8685,9 +8673,6 @@
       <c r="O53" t="n">
         <v>93278</v>
       </c>
-      <c r="Q53" t="n">
-        <v>0</v>
-      </c>
       <c r="R53" t="n">
         <v>43.67710964125839</v>
       </c>
@@ -8833,9 +8818,6 @@
       <c r="O54" t="n">
         <v>416</v>
       </c>
-      <c r="Q54" t="n">
-        <v>0</v>
-      </c>
       <c r="R54" t="n">
         <v>0.194790600256904</v>
       </c>
@@ -8981,9 +8963,6 @@
       <c r="O55" t="n">
         <v>2</v>
       </c>
-      <c r="Q55" t="n">
-        <v>0</v>
-      </c>
       <c r="R55" t="n">
         <v>0.0009364932704658844</v>
       </c>
@@ -9129,9 +9108,6 @@
       <c r="O56" t="n">
         <v>183</v>
       </c>
-      <c r="Q56" t="n">
-        <v>0</v>
-      </c>
       <c r="R56" t="n">
         <v>0.08568913424762843</v>
       </c>
@@ -9277,9 +9253,6 @@
       <c r="O57" t="n">
         <v>1780</v>
       </c>
-      <c r="Q57" t="n">
-        <v>0</v>
-      </c>
       <c r="R57" t="n">
         <v>0.8334790107146373</v>
       </c>
@@ -9425,9 +9398,6 @@
       <c r="O58" t="n">
         <v>25238</v>
       </c>
-      <c r="Q58" t="n">
-        <v>0</v>
-      </c>
       <c r="R58" t="n">
         <v>11.817608580009</v>
       </c>
@@ -9573,9 +9543,6 @@
       <c r="O59" t="n">
         <v>2</v>
       </c>
-      <c r="Q59" t="n">
-        <v>0</v>
-      </c>
       <c r="R59" t="n">
         <v>0.0009364932704658844</v>
       </c>
@@ -9721,9 +9688,6 @@
       <c r="O60" t="n">
         <v>71</v>
       </c>
-      <c r="Q60" t="n">
-        <v>0</v>
-      </c>
       <c r="R60" t="n">
         <v>0.0332455111015389</v>
       </c>
@@ -9869,9 +9833,6 @@
       <c r="O61" t="n">
         <v>87</v>
       </c>
-      <c r="Q61" t="n">
-        <v>0</v>
-      </c>
       <c r="R61" t="n">
         <v>0.04073745726526598</v>
       </c>
@@ -10017,9 +9978,6 @@
       <c r="O62" t="n">
         <v>15</v>
       </c>
-      <c r="Q62" t="n">
-        <v>0</v>
-      </c>
       <c r="R62" t="n">
         <v>0.007023699528494134</v>
       </c>
@@ -10165,9 +10123,6 @@
       <c r="O63" t="n">
         <v>3</v>
       </c>
-      <c r="Q63" t="n">
-        <v>0</v>
-      </c>
       <c r="R63" t="n">
         <v>0.001404739905698827</v>
       </c>
@@ -10313,9 +10268,6 @@
       <c r="O64" t="n">
         <v>34632</v>
       </c>
-      <c r="Q64" t="n">
-        <v>0</v>
-      </c>
       <c r="R64" t="n">
         <v>16.21631747138726</v>
       </c>
@@ -10461,9 +10413,6 @@
       <c r="O65" t="n">
         <v>50353</v>
       </c>
-      <c r="Q65" t="n">
-        <v>0</v>
-      </c>
       <c r="R65" t="n">
         <v>23.57762282388434</v>
       </c>
@@ -10609,9 +10558,6 @@
       <c r="O66" t="n">
         <v>23883</v>
       </c>
-      <c r="Q66" t="n">
-        <v>0</v>
-      </c>
       <c r="R66" t="n">
         <v>11.18313438926836</v>
       </c>
@@ -10757,9 +10703,6 @@
       <c r="O67" t="n">
         <v>14</v>
       </c>
-      <c r="Q67" t="n">
-        <v>0</v>
-      </c>
       <c r="R67" t="n">
         <v>0.006555452893261191</v>
       </c>
@@ -10905,9 +10848,6 @@
       <c r="O68" t="n">
         <v>52</v>
       </c>
-      <c r="Q68" t="n">
-        <v>0</v>
-      </c>
       <c r="R68" t="n">
         <v>0.024348825032113</v>
       </c>
@@ -11550,9 +11490,6 @@
       <c r="O71" t="n">
         <v>172</v>
       </c>
-      <c r="Q71" t="n">
-        <v>0</v>
-      </c>
       <c r="R71" t="n">
         <v>0.08053842126006606</v>
       </c>
@@ -11698,9 +11635,6 @@
       <c r="O72" t="n">
         <v>2529</v>
       </c>
-      <c r="Q72" t="n">
-        <v>0</v>
-      </c>
       <c r="R72" t="n">
         <v>1.184195740504111</v>
       </c>
@@ -11860,9 +11794,6 @@
       <c r="O73" t="n">
         <v>82988</v>
       </c>
-      <c r="Q73" t="n">
-        <v>0</v>
-      </c>
       <c r="R73" t="n">
         <v>38.85885176471141</v>
       </c>
@@ -12008,9 +11939,6 @@
       <c r="O74" t="n">
         <v>405</v>
       </c>
-      <c r="Q74" t="n">
-        <v>0</v>
-      </c>
       <c r="R74" t="n">
         <v>0.1896398872693416</v>
       </c>
@@ -12156,9 +12084,6 @@
       <c r="O75" t="n">
         <v>7</v>
       </c>
-      <c r="Q75" t="n">
-        <v>0</v>
-      </c>
       <c r="R75" t="n">
         <v>0.003277726446630596</v>
       </c>
@@ -12304,9 +12229,6 @@
       <c r="O76" t="n">
         <v>1662</v>
       </c>
-      <c r="Q76" t="n">
-        <v>0</v>
-      </c>
       <c r="R76" t="n">
         <v>0.7782259077571501</v>
       </c>
@@ -12452,9 +12374,6 @@
       <c r="O77" t="n">
         <v>95</v>
       </c>
-      <c r="Q77" t="n">
-        <v>0</v>
-      </c>
       <c r="R77" t="n">
         <v>0.04448343034712952</v>
       </c>
@@ -12600,9 +12519,6 @@
       <c r="O78" t="n">
         <v>911</v>
       </c>
-      <c r="Q78" t="n">
-        <v>0</v>
-      </c>
       <c r="R78" t="n">
         <v>0.4265726846972104</v>
       </c>
@@ -12748,9 +12664,6 @@
       <c r="O79" t="n">
         <v>1829</v>
       </c>
-      <c r="Q79" t="n">
-        <v>0</v>
-      </c>
       <c r="R79" t="n">
         <v>0.8564230958410515</v>
       </c>
@@ -12896,9 +12809,6 @@
       <c r="O80" t="n">
         <v>21823</v>
       </c>
-      <c r="Q80" t="n">
-        <v>0</v>
-      </c>
       <c r="R80" t="n">
         <v>10.2185463206885</v>
       </c>
@@ -13044,9 +12954,6 @@
       <c r="O81" t="n">
         <v>5</v>
       </c>
-      <c r="Q81" t="n">
-        <v>0</v>
-      </c>
       <c r="R81" t="n">
         <v>0.002341233176164712</v>
       </c>
@@ -13192,9 +13099,6 @@
       <c r="O82" t="n">
         <v>69</v>
       </c>
-      <c r="Q82" t="n">
-        <v>0</v>
-      </c>
       <c r="R82" t="n">
         <v>0.03230901783107301</v>
       </c>
@@ -13340,9 +13244,6 @@
       <c r="O83" t="n">
         <v>9</v>
       </c>
-      <c r="Q83" t="n">
-        <v>0</v>
-      </c>
       <c r="R83" t="n">
         <v>0.004214219717096481</v>
       </c>
@@ -13488,9 +13389,6 @@
       <c r="O84" t="n">
         <v>13</v>
       </c>
-      <c r="Q84" t="n">
-        <v>0</v>
-      </c>
       <c r="R84" t="n">
         <v>0.006087206258028249</v>
       </c>
@@ -13636,9 +13534,6 @@
       <c r="O85" t="n">
         <v>32004</v>
       </c>
-      <c r="Q85" t="n">
-        <v>0</v>
-      </c>
       <c r="R85" t="n">
         <v>14.98576531399508</v>
       </c>
@@ -13784,9 +13679,6 @@
       <c r="O86" t="n">
         <v>3073</v>
       </c>
-      <c r="Q86" t="n">
-        <v>0</v>
-      </c>
       <c r="R86" t="n">
         <v>1.438921910070831</v>
       </c>
@@ -13932,9 +13824,6 @@
       <c r="O87" t="n">
         <v>18605</v>
       </c>
-      <c r="Q87" t="n">
-        <v>0</v>
-      </c>
       <c r="R87" t="n">
         <v>8.71172864850889</v>
       </c>
@@ -14080,9 +13969,6 @@
       <c r="O88" t="n">
         <v>14419</v>
       </c>
-      <c r="Q88" t="n">
-        <v>0</v>
-      </c>
       <c r="R88" t="n">
         <v>6.751648233423794</v>
       </c>
@@ -14228,9 +14114,6 @@
       <c r="O89" t="n">
         <v>120</v>
       </c>
-      <c r="Q89" t="n">
-        <v>0</v>
-      </c>
       <c r="R89" t="n">
         <v>0.05618959622795307</v>
       </c>
@@ -14376,9 +14259,6 @@
       <c r="O90" t="n">
         <v>74</v>
       </c>
-      <c r="Q90" t="n">
-        <v>0</v>
-      </c>
       <c r="R90" t="n">
         <v>0.03465025100723772</v>
       </c>
@@ -14524,9 +14404,6 @@
       <c r="O91" t="n">
         <v>14989</v>
       </c>
-      <c r="Q91" t="n">
-        <v>0</v>
-      </c>
       <c r="R91" t="n">
         <v>7.018548815506572</v>
       </c>
@@ -14672,9 +14549,6 @@
       <c r="O92" t="n">
         <v>547</v>
       </c>
-      <c r="Q92" t="n">
-        <v>0</v>
-      </c>
       <c r="R92" t="n">
         <v>0.2561309094724194</v>
       </c>
@@ -15068,9 +14942,6 @@
       <c r="O94" t="n">
         <v>206</v>
       </c>
-      <c r="Q94" t="n">
-        <v>0</v>
-      </c>
       <c r="R94" t="n">
         <v>0.09645880685798612</v>
       </c>
@@ -15464,9 +15335,6 @@
       <c r="O96" t="n">
         <v>8</v>
       </c>
-      <c r="Q96" t="n">
-        <v>0</v>
-      </c>
       <c r="R96" t="n">
         <v>0.003745973081863538</v>
       </c>
@@ -15612,9 +15480,6 @@
       <c r="O97" t="n">
         <v>32</v>
       </c>
-      <c r="Q97" t="n">
-        <v>0</v>
-      </c>
       <c r="R97" t="n">
         <v>0.01498389232745415</v>
       </c>
@@ -15760,9 +15625,6 @@
       <c r="O98" t="n">
         <v>4</v>
       </c>
-      <c r="Q98" t="n">
-        <v>0</v>
-      </c>
       <c r="R98" t="n">
         <v>0.001872986540931769</v>
       </c>
@@ -16405,9 +16267,6 @@
       <c r="O101" t="n">
         <v>1</v>
       </c>
-      <c r="Q101" t="n">
-        <v>0</v>
-      </c>
       <c r="R101" t="n">
         <v>0.0004682466352329422</v>
       </c>
@@ -16553,9 +16412,6 @@
       <c r="O102" t="n">
         <v>2268</v>
       </c>
-      <c r="Q102" t="n">
-        <v>0</v>
-      </c>
       <c r="R102" t="n">
         <v>1.061983368708313</v>
       </c>
@@ -16715,9 +16571,6 @@
       <c r="O103" t="n">
         <v>59160</v>
       </c>
-      <c r="Q103" t="n">
-        <v>0</v>
-      </c>
       <c r="R103" t="n">
         <v>27.70147094038087</v>
       </c>
@@ -16863,9 +16716,6 @@
       <c r="O104" t="n">
         <v>375</v>
       </c>
-      <c r="Q104" t="n">
-        <v>0</v>
-      </c>
       <c r="R104" t="n">
         <v>0.1755924882123533</v>
       </c>
@@ -17011,9 +16861,6 @@
       <c r="O105" t="n">
         <v>731</v>
       </c>
-      <c r="Q105" t="n">
-        <v>0</v>
-      </c>
       <c r="R105" t="n">
         <v>0.3422882903552808</v>
       </c>
@@ -17159,9 +17006,6 @@
       <c r="O106" t="n">
         <v>1459</v>
       </c>
-      <c r="Q106" t="n">
-        <v>0</v>
-      </c>
       <c r="R106" t="n">
         <v>0.6831718408048627</v>
       </c>
@@ -17307,9 +17151,6 @@
       <c r="O107" t="n">
         <v>13282</v>
       </c>
-      <c r="Q107" t="n">
-        <v>0</v>
-      </c>
       <c r="R107" t="n">
         <v>6.219251809163939</v>
       </c>
@@ -17455,9 +17296,6 @@
       <c r="O108" t="n">
         <v>71</v>
       </c>
-      <c r="Q108" t="n">
-        <v>0</v>
-      </c>
       <c r="R108" t="n">
         <v>0.0332455111015389</v>
       </c>
@@ -17603,9 +17441,6 @@
       <c r="O109" t="n">
         <v>16945</v>
       </c>
-      <c r="Q109" t="n">
-        <v>0</v>
-      </c>
       <c r="R109" t="n">
         <v>7.934439234022207</v>
       </c>
@@ -17751,9 +17586,6 @@
       <c r="O110" t="n">
         <v>20949</v>
       </c>
-      <c r="Q110" t="n">
-        <v>0</v>
-      </c>
       <c r="R110" t="n">
         <v>9.809298761494908</v>
       </c>
@@ -17899,9 +17731,6 @@
       <c r="O111" t="n">
         <v>1397</v>
       </c>
-      <c r="Q111" t="n">
-        <v>0</v>
-      </c>
       <c r="R111" t="n">
         <v>0.6541405494204203</v>
       </c>
@@ -18295,9 +18124,6 @@
       <c r="O113" t="n">
         <v>40053</v>
       </c>
-      <c r="Q113" t="n">
-        <v>0</v>
-      </c>
       <c r="R113" t="n">
         <v>18.75468248098504</v>
       </c>
@@ -18443,9 +18269,6 @@
       <c r="O114" t="n">
         <v>219</v>
       </c>
-      <c r="Q114" t="n">
-        <v>0</v>
-      </c>
       <c r="R114" t="n">
         <v>0.1025460131160144</v>
       </c>
@@ -18591,9 +18414,6 @@
       <c r="O115" t="n">
         <v>1</v>
       </c>
-      <c r="Q115" t="n">
-        <v>0</v>
-      </c>
       <c r="R115" t="n">
         <v>0.0004682466352329422</v>
       </c>
@@ -18739,9 +18559,6 @@
       <c r="O116" t="n">
         <v>2</v>
       </c>
-      <c r="Q116" t="n">
-        <v>0</v>
-      </c>
       <c r="R116" t="n">
         <v>0.0009364932704658844</v>
       </c>
@@ -18887,9 +18704,6 @@
       <c r="O117" t="n">
         <v>461</v>
       </c>
-      <c r="Q117" t="n">
-        <v>0</v>
-      </c>
       <c r="R117" t="n">
         <v>0.2158616988423864</v>
       </c>
@@ -19035,9 +18849,6 @@
       <c r="O118" t="n">
         <v>8040</v>
       </c>
-      <c r="Q118" t="n">
-        <v>0</v>
-      </c>
       <c r="R118" t="n">
         <v>3.764702947272856</v>
       </c>
@@ -19183,9 +18994,6 @@
       <c r="O119" t="n">
         <v>49</v>
       </c>
-      <c r="Q119" t="n">
-        <v>0</v>
-      </c>
       <c r="R119" t="n">
         <v>0.02294408512641417</v>
       </c>
@@ -19331,9 +19139,6 @@
       <c r="O120" t="n">
         <v>257</v>
       </c>
-      <c r="Q120" t="n">
-        <v>0</v>
-      </c>
       <c r="R120" t="n">
         <v>0.1203393852548662</v>
       </c>
@@ -19479,9 +19284,6 @@
       <c r="O121" t="n">
         <v>10172</v>
       </c>
-      <c r="Q121" t="n">
-        <v>0</v>
-      </c>
       <c r="R121" t="n">
         <v>4.763004773589489</v>
       </c>
@@ -19627,9 +19429,6 @@
       <c r="O122" t="n">
         <v>9</v>
       </c>
-      <c r="Q122" t="n">
-        <v>0</v>
-      </c>
       <c r="R122" t="n">
         <v>0.004214219717096481</v>
       </c>
@@ -20023,9 +19822,6 @@
       <c r="O124" t="n">
         <v>101</v>
       </c>
-      <c r="Q124" t="n">
-        <v>0</v>
-      </c>
       <c r="R124" t="n">
         <v>0.04729291015852717</v>
       </c>
@@ -20171,9 +19967,6 @@
       <c r="O125" t="n">
         <v>11</v>
       </c>
-      <c r="Q125" t="n">
-        <v>0</v>
-      </c>
       <c r="R125" t="n">
         <v>0.005150712987562365</v>
       </c>
@@ -20318,9 +20111,6 @@
       </c>
       <c r="O126" t="n">
         <v>1</v>
-      </c>
-      <c r="Q126" t="n">
-        <v>0</v>
       </c>
       <c r="R126" t="n">
         <v>0.0004682466352329422</v>

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-23 02:00:45 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -16566,13 +16566,13 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>59160</v>
+        <v>54138</v>
       </c>
       <c r="O103" t="n">
-        <v>59160</v>
+        <v>54138</v>
       </c>
       <c r="R103" t="n">
-        <v>27.70147094038087</v>
+        <v>25.34993633824103</v>
       </c>
       <c r="S103" t="inlineStr">
         <is>
@@ -17001,13 +17001,13 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>1459</v>
+        <v>1542</v>
       </c>
       <c r="O106" t="n">
-        <v>1459</v>
+        <v>1542</v>
       </c>
       <c r="R106" t="n">
-        <v>0.6831718408048627</v>
+        <v>0.722036311529197</v>
       </c>
       <c r="S106" t="inlineStr">
         <is>
@@ -17146,13 +17146,13 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>13282</v>
+        <v>13777</v>
       </c>
       <c r="O107" t="n">
-        <v>13282</v>
+        <v>13777</v>
       </c>
       <c r="R107" t="n">
-        <v>6.219251809163939</v>
+        <v>6.451033893604246</v>
       </c>
       <c r="S107" t="inlineStr">
         <is>
@@ -17726,13 +17726,13 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>1397</v>
+        <v>2489</v>
       </c>
       <c r="O111" t="n">
-        <v>1397</v>
+        <v>2489</v>
       </c>
       <c r="R111" t="n">
-        <v>0.6541405494204203</v>
+        <v>1.165465875094793</v>
       </c>
       <c r="S111" t="inlineStr">
         <is>
@@ -17885,10 +17885,10 @@
         </is>
       </c>
       <c r="N112" t="n">
-        <v>1397</v>
+        <v>2489</v>
       </c>
       <c r="O112" t="n">
-        <v>1397</v>
+        <v>2489</v>
       </c>
       <c r="U112" t="inlineStr">
         <is>
@@ -18119,13 +18119,13 @@
         </is>
       </c>
       <c r="N113" t="n">
-        <v>40053</v>
+        <v>46395</v>
       </c>
       <c r="O113" t="n">
-        <v>40053</v>
+        <v>46395</v>
       </c>
       <c r="R113" t="n">
-        <v>18.75468248098504</v>
+        <v>21.72430264163236</v>
       </c>
       <c r="S113" t="inlineStr">
         <is>
@@ -18699,13 +18699,13 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>461</v>
+        <v>989</v>
       </c>
       <c r="O117" t="n">
-        <v>461</v>
+        <v>989</v>
       </c>
       <c r="R117" t="n">
-        <v>0.2158616988423864</v>
+        <v>0.4630959222453799</v>
       </c>
       <c r="S117" t="inlineStr">
         <is>
@@ -18844,13 +18844,13 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>8040</v>
+        <v>10364</v>
       </c>
       <c r="O118" t="n">
-        <v>8040</v>
+        <v>10364</v>
       </c>
       <c r="R118" t="n">
-        <v>3.764702947272856</v>
+        <v>4.852908127554214</v>
       </c>
       <c r="S118" t="inlineStr">
         <is>
@@ -19424,13 +19424,13 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>9</v>
+        <v>1597</v>
       </c>
       <c r="O122" t="n">
-        <v>9</v>
+        <v>1597</v>
       </c>
       <c r="R122" t="n">
-        <v>0.004214219717096481</v>
+        <v>0.7477898764670088</v>
       </c>
       <c r="S122" t="inlineStr">
         <is>
@@ -19583,10 +19583,10 @@
         </is>
       </c>
       <c r="N123" t="n">
-        <v>9</v>
+        <v>1597</v>
       </c>
       <c r="O123" t="n">
-        <v>9</v>
+        <v>1597</v>
       </c>
       <c r="U123" t="inlineStr">
         <is>
@@ -19817,13 +19817,13 @@
         </is>
       </c>
       <c r="N124" t="n">
-        <v>101</v>
+        <v>18558</v>
       </c>
       <c r="O124" t="n">
-        <v>101</v>
+        <v>18558</v>
       </c>
       <c r="R124" t="n">
-        <v>0.04729291015852717</v>
+        <v>8.689721056652942</v>
       </c>
       <c r="S124" t="inlineStr">
         <is>
@@ -19933,17 +19933,17 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -19962,13 +19962,13 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="O125" t="n">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="R125" t="n">
-        <v>0.005150712987562365</v>
+        <v>0.009833179339891788</v>
       </c>
       <c r="S125" t="inlineStr">
         <is>
@@ -20078,22 +20078,22 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
@@ -20107,13 +20107,13 @@
         </is>
       </c>
       <c r="N126" t="n">
-        <v>1</v>
+        <v>2432</v>
       </c>
       <c r="O126" t="n">
-        <v>1</v>
+        <v>2432</v>
       </c>
       <c r="R126" t="n">
-        <v>0.0004682466352329422</v>
+        <v>1.138775816886516</v>
       </c>
       <c r="S126" t="inlineStr">
         <is>
@@ -20180,6 +20180,544 @@
         </is>
       </c>
       <c r="BC126" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>D120</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>破伤风</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N127" t="n">
+        <v>1</v>
+      </c>
+      <c r="O127" t="n">
+        <v>1</v>
+      </c>
+      <c r="R127" t="n">
+        <v>0.0004682466352329422</v>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO127" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP127" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR127" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS127" t="inlineStr"/>
+      <c r="AT127" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU127" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV127" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW127" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX127" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY127" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ127" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA127" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB127" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC127" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N128" t="n">
+        <v>10</v>
+      </c>
+      <c r="O128" t="n">
+        <v>10</v>
+      </c>
+      <c r="R128" t="n">
+        <v>0.004682466352329423</v>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA128" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO128" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP128" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ128" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS128" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT128" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU128" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV128" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW128" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX128" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY128" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ128" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA128" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB128" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC128" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N129" t="n">
+        <v>10</v>
+      </c>
+      <c r="O129" t="n">
+        <v>10</v>
+      </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W129" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X129" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y129" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z129" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA129" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC129" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD129" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE129" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF129" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG129" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH129" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI129" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ129" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK129" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM129" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN129" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO129" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP129" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ129" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS129" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT129" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU129" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV129" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW129" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX129" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY129" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ129" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA129" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB129" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC129" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -20301,7 +20839,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10">
@@ -20311,7 +20849,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11">
@@ -20331,7 +20869,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -20363,7 +20901,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1013060</v>
+        <v>1041399</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-27 08:21:19 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -16566,13 +16566,13 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>54138</v>
+        <v>53049</v>
       </c>
       <c r="O103" t="n">
-        <v>54138</v>
+        <v>53049</v>
       </c>
       <c r="R103" t="n">
-        <v>25.34993633824103</v>
+        <v>24.84001575247235</v>
       </c>
       <c r="S103" t="inlineStr">
         <is>
@@ -17001,13 +17001,13 @@
         </is>
       </c>
       <c r="N106" t="n">
-        <v>1542</v>
+        <v>1593</v>
       </c>
       <c r="O106" t="n">
-        <v>1542</v>
+        <v>1593</v>
       </c>
       <c r="R106" t="n">
-        <v>0.722036311529197</v>
+        <v>0.7459168899260771</v>
       </c>
       <c r="S106" t="inlineStr">
         <is>
@@ -17146,13 +17146,13 @@
         </is>
       </c>
       <c r="N107" t="n">
-        <v>13777</v>
+        <v>13901</v>
       </c>
       <c r="O107" t="n">
-        <v>13777</v>
+        <v>13901</v>
       </c>
       <c r="R107" t="n">
-        <v>6.451033893604246</v>
+        <v>6.509096476373131</v>
       </c>
       <c r="S107" t="inlineStr">
         <is>
@@ -17407,17 +17407,17 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -17436,13 +17436,13 @@
         </is>
       </c>
       <c r="N109" t="n">
-        <v>16945</v>
+        <v>32</v>
       </c>
       <c r="O109" t="n">
-        <v>16945</v>
+        <v>32</v>
       </c>
       <c r="R109" t="n">
-        <v>7.934439234022207</v>
+        <v>0.01498389232745415</v>
       </c>
       <c r="S109" t="inlineStr">
         <is>
@@ -17552,17 +17552,17 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>D191</t>
+          <t>D184</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Exogenous poisoning</t>
+          <t>Accident caused by venomous animals</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>外源性中毒</t>
+          <t>毒性动物伤害</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -17581,13 +17581,13 @@
         </is>
       </c>
       <c r="N110" t="n">
-        <v>20949</v>
+        <v>27520</v>
       </c>
       <c r="O110" t="n">
-        <v>20949</v>
+        <v>27520</v>
       </c>
       <c r="R110" t="n">
-        <v>9.809298761494908</v>
+        <v>12.88614740161057</v>
       </c>
       <c r="S110" t="inlineStr">
         <is>
@@ -17697,17 +17697,17 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D191</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Exogenous poisoning</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>外源性中毒</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -17726,55 +17726,41 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>2489</v>
+        <v>20949</v>
       </c>
       <c r="O111" t="n">
-        <v>2489</v>
+        <v>20949</v>
       </c>
       <c r="R111" t="n">
-        <v>1.165465875094793</v>
+        <v>9.809298761494908</v>
       </c>
       <c r="S111" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA111" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO111" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP111" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ111" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS111" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR111" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS111" t="inlineStr"/>
       <c r="AT111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU111" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV111" t="inlineStr">
@@ -17841,7 +17827,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -17890,98 +17876,23 @@
       <c r="O112" t="n">
         <v>2489</v>
       </c>
+      <c r="R112" t="n">
+        <v>1.165465875094793</v>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U112" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="V112" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W112" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X112" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y112" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z112" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA112" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB112" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC112" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD112" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE112" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF112" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG112" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH112" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI112" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ112" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK112" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM112" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN112" t="b">
-        <v>1</v>
       </c>
       <c r="AO112" t="inlineStr">
         <is>
@@ -18075,7 +17986,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -18090,70 +18001,159 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="N113" t="n">
-        <v>46395</v>
+        <v>2489</v>
       </c>
       <c r="O113" t="n">
-        <v>46395</v>
-      </c>
-      <c r="R113" t="n">
-        <v>21.72430264163236</v>
-      </c>
-      <c r="S113" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>2489</v>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA113" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB113" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC113" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD113" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE113" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF113" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG113" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH113" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI113" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ113" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK113" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM113" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN113" t="b">
+        <v>1</v>
       </c>
       <c r="AO113" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP113" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR113" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS113" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ113" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS113" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU113" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV113" t="inlineStr">
@@ -18235,22 +18235,22 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>D028</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>百日咳</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -18264,13 +18264,13 @@
         </is>
       </c>
       <c r="N114" t="n">
-        <v>219</v>
+        <v>44692</v>
       </c>
       <c r="O114" t="n">
-        <v>219</v>
+        <v>44692</v>
       </c>
       <c r="R114" t="n">
-        <v>0.1025460131160144</v>
+        <v>20.92687862183066</v>
       </c>
       <c r="S114" t="inlineStr">
         <is>
@@ -18380,17 +18380,17 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -18409,13 +18409,13 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>1</v>
+        <v>219</v>
       </c>
       <c r="O115" t="n">
-        <v>1</v>
+        <v>219</v>
       </c>
       <c r="R115" t="n">
-        <v>0.0004682466352329422</v>
+        <v>0.1025460131160144</v>
       </c>
       <c r="S115" t="inlineStr">
         <is>
@@ -18525,17 +18525,17 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>D035</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Leptospirosis</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>钩端螺旋体病</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -18554,13 +18554,13 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R116" t="n">
-        <v>0.0009364932704658844</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S116" t="inlineStr">
         <is>
@@ -18670,22 +18670,22 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D035</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Leptospirosis</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>钩端螺旋体病</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -18699,13 +18699,13 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>989</v>
+        <v>2</v>
       </c>
       <c r="O117" t="n">
-        <v>989</v>
+        <v>2</v>
       </c>
       <c r="R117" t="n">
-        <v>0.4630959222453799</v>
+        <v>0.0009364932704658844</v>
       </c>
       <c r="S117" t="inlineStr">
         <is>
@@ -18815,17 +18815,17 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -18844,13 +18844,13 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>10364</v>
+        <v>1169</v>
       </c>
       <c r="O118" t="n">
-        <v>10364</v>
+        <v>1169</v>
       </c>
       <c r="R118" t="n">
-        <v>4.852908127554214</v>
+        <v>0.5473803165873095</v>
       </c>
       <c r="S118" t="inlineStr">
         <is>
@@ -18960,22 +18960,22 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -18989,13 +18989,13 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>49</v>
+        <v>10988</v>
       </c>
       <c r="O119" t="n">
-        <v>49</v>
+        <v>10988</v>
       </c>
       <c r="R119" t="n">
-        <v>0.02294408512641417</v>
+        <v>5.14509402793957</v>
       </c>
       <c r="S119" t="inlineStr">
         <is>
@@ -19105,22 +19105,22 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -19134,13 +19134,13 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>257</v>
+        <v>49</v>
       </c>
       <c r="O120" t="n">
-        <v>257</v>
+        <v>49</v>
       </c>
       <c r="R120" t="n">
-        <v>0.1203393852548662</v>
+        <v>0.02294408512641417</v>
       </c>
       <c r="S120" t="inlineStr">
         <is>
@@ -19250,17 +19250,17 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>D191</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Exogenous poisoning</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>外源性中毒</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -19279,13 +19279,13 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>10172</v>
+        <v>38</v>
       </c>
       <c r="O121" t="n">
-        <v>10172</v>
+        <v>38</v>
       </c>
       <c r="R121" t="n">
-        <v>4.763004773589489</v>
+        <v>0.01779337213885181</v>
       </c>
       <c r="S121" t="inlineStr">
         <is>
@@ -19395,17 +19395,17 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D184</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Accident caused by venomous animals</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>毒性动物伤害</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -19424,55 +19424,41 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>1597</v>
+        <v>26801</v>
       </c>
       <c r="O122" t="n">
-        <v>1597</v>
+        <v>26801</v>
       </c>
       <c r="R122" t="n">
-        <v>0.7477898764670088</v>
+        <v>12.54947807087809</v>
       </c>
       <c r="S122" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA122" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO122" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP122" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ122" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS122" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR122" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS122" t="inlineStr"/>
       <c r="AT122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU122" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV122" t="inlineStr">
@@ -19539,7 +19525,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -19554,17 +19540,17 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D191</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Exogenous poisoning</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>外源性中毒</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -19583,130 +19569,41 @@
         </is>
       </c>
       <c r="N123" t="n">
-        <v>1597</v>
+        <v>10172</v>
       </c>
       <c r="O123" t="n">
-        <v>1597</v>
-      </c>
-      <c r="U123" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="V123" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W123" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X123" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y123" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z123" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="AA123" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="AB123" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC123" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD123" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE123" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF123" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG123" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH123" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI123" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ123" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK123" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM123" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN123" t="b">
-        <v>1</v>
+        <v>10172</v>
+      </c>
+      <c r="R123" t="n">
+        <v>4.763004773589489</v>
+      </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
       </c>
       <c r="AO123" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP123" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ123" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS123" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR123" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS123" t="inlineStr"/>
       <c r="AT123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU123" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV123" t="inlineStr">
@@ -19788,70 +19685,84 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N124" t="n">
-        <v>18558</v>
+        <v>1597</v>
       </c>
       <c r="O124" t="n">
-        <v>18558</v>
+        <v>1597</v>
       </c>
       <c r="R124" t="n">
-        <v>8.689721056652942</v>
+        <v>0.7477898764670088</v>
       </c>
       <c r="S124" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA124" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO124" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP124" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR124" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS124" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ124" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS124" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU124" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV124" t="inlineStr">
@@ -19918,7 +19829,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -19933,70 +19844,159 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M125" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N125" t="n">
-        <v>21</v>
+        <v>1597</v>
       </c>
       <c r="O125" t="n">
-        <v>21</v>
-      </c>
-      <c r="R125" t="n">
-        <v>0.009833179339891788</v>
-      </c>
-      <c r="S125" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>1597</v>
+      </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W125" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA125" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB125" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC125" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD125" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE125" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF125" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG125" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH125" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI125" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ125" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK125" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM125" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN125" t="b">
+        <v>1</v>
       </c>
       <c r="AO125" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP125" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR125" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS125" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ125" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS125" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT125" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU125" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV125" t="inlineStr">
@@ -20078,17 +20078,17 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -20107,13 +20107,13 @@
         </is>
       </c>
       <c r="N126" t="n">
-        <v>2432</v>
+        <v>28051</v>
       </c>
       <c r="O126" t="n">
-        <v>2432</v>
+        <v>28051</v>
       </c>
       <c r="R126" t="n">
-        <v>1.138775816886516</v>
+        <v>13.13478636491926</v>
       </c>
       <c r="S126" t="inlineStr">
         <is>
@@ -20223,22 +20223,22 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -20252,13 +20252,13 @@
         </is>
       </c>
       <c r="N127" t="n">
-        <v>1</v>
+        <v>96</v>
       </c>
       <c r="O127" t="n">
-        <v>1</v>
+        <v>96</v>
       </c>
       <c r="R127" t="n">
-        <v>0.0004682466352329422</v>
+        <v>0.04495167698236246</v>
       </c>
       <c r="S127" t="inlineStr">
         <is>
@@ -20368,22 +20368,22 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
@@ -20397,55 +20397,41 @@
         </is>
       </c>
       <c r="N128" t="n">
-        <v>10</v>
+        <v>4202</v>
       </c>
       <c r="O128" t="n">
-        <v>10</v>
+        <v>4202</v>
       </c>
       <c r="R128" t="n">
-        <v>0.004682466352329423</v>
+        <v>1.967572361248823</v>
       </c>
       <c r="S128" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U128" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA128" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO128" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP128" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ128" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS128" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR128" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS128" t="inlineStr"/>
       <c r="AT128" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU128" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV128" t="inlineStr">
@@ -20512,212 +20498,806 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>D120</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Tetanus</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>破伤风</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N129" t="n">
+        <v>1</v>
+      </c>
+      <c r="O129" t="n">
+        <v>1</v>
+      </c>
+      <c r="R129" t="n">
+        <v>0.0004682466352329422</v>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO129" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP129" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR129" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS129" t="inlineStr"/>
+      <c r="AT129" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU129" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV129" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW129" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX129" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY129" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ129" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA129" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB129" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC129" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>D178</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Acute flaccid paralysis</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>急性无力肢体麻痹</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N130" t="n">
+        <v>1</v>
+      </c>
+      <c r="O130" t="n">
+        <v>1</v>
+      </c>
+      <c r="R130" t="n">
+        <v>0.0004682466352329422</v>
+      </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO130" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP130" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR130" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS130" t="inlineStr"/>
+      <c r="AT130" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU130" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV130" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW130" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX130" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY130" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ130" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA130" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB130" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC130" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>D184</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Accident caused by venomous animals</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>毒性动物伤害</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N131" t="n">
+        <v>2970</v>
+      </c>
+      <c r="O131" t="n">
+        <v>2970</v>
+      </c>
+      <c r="R131" t="n">
+        <v>1.390692506641839</v>
+      </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO131" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP131" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR131" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS131" t="inlineStr"/>
+      <c r="AT131" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU131" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV131" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW131" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX131" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY131" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ131" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA131" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB131" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC131" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N132" t="n">
+        <v>10</v>
+      </c>
+      <c r="O132" t="n">
+        <v>10</v>
+      </c>
+      <c r="R132" t="n">
+        <v>0.004682466352329423</v>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA132" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO132" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP132" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ132" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS132" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT132" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU132" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV132" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW132" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX132" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY132" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ132" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA132" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB132" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC132" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
           <t>source_series_observation</t>
         </is>
       </c>
-      <c r="F129" t="inlineStr">
+      <c r="F133" t="inlineStr">
         <is>
           <t>BR</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr">
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
         <is>
           <t>D235</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr">
+      <c r="I133" t="inlineStr">
         <is>
           <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr">
+      <c r="J133" t="inlineStr">
         <is>
           <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr">
+      <c r="K133" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L129" t="inlineStr">
+      <c r="L133" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="M129" t="inlineStr">
+      <c r="M133" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="N129" t="n">
+      <c r="N133" t="n">
         <v>10</v>
       </c>
-      <c r="O129" t="n">
+      <c r="O133" t="n">
         <v>10</v>
       </c>
-      <c r="U129" t="inlineStr">
+      <c r="U133" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="V129" t="inlineStr">
+      <c r="V133" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="W129" t="inlineStr">
+      <c r="W133" t="inlineStr">
         <is>
           <t>SRC_BR_SINAN</t>
         </is>
       </c>
-      <c r="X129" t="inlineStr">
+      <c r="X133" t="inlineStr">
         <is>
           <t>Meningitis</t>
         </is>
       </c>
-      <c r="Y129" t="inlineStr">
+      <c r="Y133" t="inlineStr">
         <is>
           <t>case_notifications</t>
         </is>
       </c>
-      <c r="Z129" t="inlineStr">
+      <c r="Z133" t="inlineStr">
         <is>
           <t>notification</t>
         </is>
       </c>
-      <c r="AA129" t="inlineStr">
+      <c r="AA133" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="AB129" t="inlineStr">
+      <c r="AB133" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="AC129" t="inlineStr">
+      <c r="AC133" t="inlineStr">
         <is>
           <t>country:BR:national</t>
         </is>
       </c>
-      <c r="AD129" t="inlineStr">
+      <c r="AD133" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="AE129" t="inlineStr">
+      <c r="AE133" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="AF129" t="inlineStr">
+      <c r="AF133" t="inlineStr">
         <is>
           <t>conditional</t>
         </is>
       </c>
-      <c r="AG129" t="inlineStr">
+      <c r="AG133" t="inlineStr">
         <is>
           <t>reported_aggregate</t>
         </is>
       </c>
-      <c r="AH129" t="inlineStr">
+      <c r="AH133" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="AI129" t="inlineStr">
+      <c r="AI133" t="inlineStr">
         <is>
           <t>missing_is_unknown</t>
         </is>
       </c>
-      <c r="AJ129" t="inlineStr">
+      <c r="AJ133" t="inlineStr">
         <is>
           <t>BR_SINAN_MENI_current</t>
         </is>
       </c>
-      <c r="AK129" t="inlineStr">
+      <c r="AK133" t="inlineStr">
         <is>
           <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
         </is>
       </c>
-      <c r="AM129" t="inlineStr">
+      <c r="AM133" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>
       </c>
-      <c r="AN129" t="b">
+      <c r="AN133" t="b">
         <v>1</v>
       </c>
-      <c r="AO129" t="inlineStr">
+      <c r="AO133" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
       </c>
-      <c r="AP129" t="inlineStr">
+      <c r="AP133" t="inlineStr">
         <is>
           <t>single_series</t>
         </is>
       </c>
-      <c r="AQ129" t="inlineStr">
+      <c r="AQ133" t="inlineStr">
         <is>
           <t>legacy_gap_fill</t>
         </is>
       </c>
-      <c r="AS129" t="inlineStr">
+      <c r="AS133" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="AT129" t="n">
+      <c r="AT133" t="n">
         <v>1</v>
       </c>
-      <c r="AU129" t="inlineStr">
+      <c r="AU133" t="inlineStr">
         <is>
           <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
-      <c r="AV129" t="inlineStr">
-        <is>
-          <t>sinan_datasus</t>
-        </is>
-      </c>
-      <c r="AW129" t="inlineStr">
-        <is>
-          <t>Brazil DATASUS SINAN</t>
-        </is>
-      </c>
-      <c r="AX129" t="inlineStr">
-        <is>
-          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
-        </is>
-      </c>
-      <c r="AY129" t="inlineStr">
-        <is>
-          <t>ftp_dbc</t>
-        </is>
-      </c>
-      <c r="AZ129" t="inlineStr">
-        <is>
-          <t>sinan_datasus</t>
-        </is>
-      </c>
-      <c r="BA129" t="inlineStr">
-        <is>
-          <t>Brazil DATASUS SINAN</t>
-        </is>
-      </c>
-      <c r="BB129" t="inlineStr">
-        <is>
-          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
-        </is>
-      </c>
-      <c r="BC129" t="inlineStr">
+      <c r="AV133" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW133" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX133" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY133" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ133" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA133" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB133" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC133" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -20839,7 +21419,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10">
@@ -20849,7 +21429,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11">
@@ -20901,7 +21481,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1041399</v>
+        <v>1091084</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-28 12:40:05 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -3078,7 +3078,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK33" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
@@ -11089,7 +11089,7 @@
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK69" t="inlineStr">
@@ -11328,7 +11328,7 @@
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK70" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK93" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK95" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK99" t="inlineStr">
@@ -16105,7 +16105,7 @@
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.10</t>
+          <t>globalid-disease-ontology:2026.08.28</t>
         </is>
       </c>
       <c r="AK100" t="inlineStr">
@@ -17262,17 +17262,17 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D118</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Spotted fever rickettsiosis</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>斑点热立克次体病</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -17291,13 +17291,13 @@
         </is>
       </c>
       <c r="N108" t="n">
-        <v>71</v>
+        <v>344</v>
       </c>
       <c r="O108" t="n">
-        <v>71</v>
+        <v>344</v>
       </c>
       <c r="R108" t="n">
-        <v>0.0332455111015389</v>
+        <v>0.1610768425201321</v>
       </c>
       <c r="S108" t="inlineStr">
         <is>
@@ -17407,22 +17407,22 @@
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -17436,13 +17436,13 @@
         </is>
       </c>
       <c r="N109" t="n">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="O109" t="n">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="R109" t="n">
-        <v>0.01498389232745415</v>
+        <v>0.0332455111015389</v>
       </c>
       <c r="S109" t="inlineStr">
         <is>
@@ -17552,17 +17552,17 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -17581,13 +17581,13 @@
         </is>
       </c>
       <c r="N110" t="n">
-        <v>27520</v>
+        <v>32</v>
       </c>
       <c r="O110" t="n">
-        <v>27520</v>
+        <v>32</v>
       </c>
       <c r="R110" t="n">
-        <v>12.88614740161057</v>
+        <v>0.01498389232745415</v>
       </c>
       <c r="S110" t="inlineStr">
         <is>
@@ -17697,17 +17697,17 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>D191</t>
+          <t>D184</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Exogenous poisoning</t>
+          <t>Accident caused by venomous animals</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>外源性中毒</t>
+          <t>毒性动物伤害</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -17726,13 +17726,13 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>20949</v>
+        <v>27520</v>
       </c>
       <c r="O111" t="n">
-        <v>20949</v>
+        <v>27520</v>
       </c>
       <c r="R111" t="n">
-        <v>9.809298761494908</v>
+        <v>12.88614740161057</v>
       </c>
       <c r="S111" t="inlineStr">
         <is>
@@ -17842,17 +17842,17 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D191</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Exogenous poisoning</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>外源性中毒</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -17871,55 +17871,41 @@
         </is>
       </c>
       <c r="N112" t="n">
-        <v>2489</v>
+        <v>20949</v>
       </c>
       <c r="O112" t="n">
-        <v>2489</v>
+        <v>20949</v>
       </c>
       <c r="R112" t="n">
-        <v>1.165465875094793</v>
+        <v>9.809298761494908</v>
       </c>
       <c r="S112" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA112" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO112" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP112" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ112" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS112" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR112" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS112" t="inlineStr"/>
       <c r="AT112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU112" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV112" t="inlineStr">
@@ -17986,7 +17972,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -18035,98 +18021,23 @@
       <c r="O113" t="n">
         <v>2489</v>
       </c>
+      <c r="R113" t="n">
+        <v>1.165465875094793</v>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U113" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="V113" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W113" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X113" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y113" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z113" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA113" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB113" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC113" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD113" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE113" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF113" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG113" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH113" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI113" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ113" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK113" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM113" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN113" t="b">
-        <v>1</v>
       </c>
       <c r="AO113" t="inlineStr">
         <is>
@@ -18220,7 +18131,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -18235,70 +18146,159 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="N114" t="n">
-        <v>44692</v>
+        <v>2489</v>
       </c>
       <c r="O114" t="n">
-        <v>44692</v>
-      </c>
-      <c r="R114" t="n">
-        <v>20.92687862183066</v>
-      </c>
-      <c r="S114" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>2489</v>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA114" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB114" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC114" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD114" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE114" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF114" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG114" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH114" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI114" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ114" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK114" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM114" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN114" t="b">
+        <v>1</v>
       </c>
       <c r="AO114" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP114" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR114" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS114" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ114" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS114" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT114" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU114" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV114" t="inlineStr">
@@ -18380,22 +18380,22 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>D028</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Pertussis</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>百日咳</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
@@ -18409,13 +18409,13 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>219</v>
+        <v>44692</v>
       </c>
       <c r="O115" t="n">
-        <v>219</v>
+        <v>44692</v>
       </c>
       <c r="R115" t="n">
-        <v>0.1025460131160144</v>
+        <v>20.92687862183066</v>
       </c>
       <c r="S115" t="inlineStr">
         <is>
@@ -18525,17 +18525,17 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>D029</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Diphtheria</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>白喉</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -18554,13 +18554,13 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>1</v>
+        <v>219</v>
       </c>
       <c r="O116" t="n">
-        <v>1</v>
+        <v>219</v>
       </c>
       <c r="R116" t="n">
-        <v>0.0004682466352329422</v>
+        <v>0.1025460131160144</v>
       </c>
       <c r="S116" t="inlineStr">
         <is>
@@ -18670,17 +18670,17 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>D035</t>
+          <t>D029</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Leptospirosis</t>
+          <t>Diphtheria</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>钩端螺旋体病</t>
+          <t>白喉</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -18699,13 +18699,13 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O117" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R117" t="n">
-        <v>0.0009364932704658844</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S117" t="inlineStr">
         <is>
@@ -18815,22 +18815,22 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D035</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Leptospirosis</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>钩端螺旋体病</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -18844,13 +18844,13 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1169</v>
+        <v>2</v>
       </c>
       <c r="O118" t="n">
-        <v>1169</v>
+        <v>2</v>
       </c>
       <c r="R118" t="n">
-        <v>0.5473803165873095</v>
+        <v>0.0009364932704658844</v>
       </c>
       <c r="S118" t="inlineStr">
         <is>
@@ -18960,17 +18960,17 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -18989,13 +18989,13 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>10988</v>
+        <v>1169</v>
       </c>
       <c r="O119" t="n">
-        <v>10988</v>
+        <v>1169</v>
       </c>
       <c r="R119" t="n">
-        <v>5.14509402793957</v>
+        <v>0.5473803165873095</v>
       </c>
       <c r="S119" t="inlineStr">
         <is>
@@ -19105,22 +19105,22 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -19134,13 +19134,13 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>49</v>
+        <v>10988</v>
       </c>
       <c r="O120" t="n">
-        <v>49</v>
+        <v>10988</v>
       </c>
       <c r="R120" t="n">
-        <v>0.02294408512641417</v>
+        <v>5.14509402793957</v>
       </c>
       <c r="S120" t="inlineStr">
         <is>
@@ -19250,22 +19250,22 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D118</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Spotted fever rickettsiosis</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>斑点热立克次体病</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -19279,13 +19279,13 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="O121" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="R121" t="n">
-        <v>0.01779337213885181</v>
+        <v>0.003745973081863538</v>
       </c>
       <c r="S121" t="inlineStr">
         <is>
@@ -19395,22 +19395,22 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -19424,13 +19424,13 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>26801</v>
+        <v>49</v>
       </c>
       <c r="O122" t="n">
-        <v>26801</v>
+        <v>49</v>
       </c>
       <c r="R122" t="n">
-        <v>12.54947807087809</v>
+        <v>0.02294408512641417</v>
       </c>
       <c r="S122" t="inlineStr">
         <is>
@@ -19540,17 +19540,17 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>D191</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Exogenous poisoning</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>外源性中毒</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -19569,13 +19569,13 @@
         </is>
       </c>
       <c r="N123" t="n">
-        <v>10172</v>
+        <v>38</v>
       </c>
       <c r="O123" t="n">
-        <v>10172</v>
+        <v>38</v>
       </c>
       <c r="R123" t="n">
-        <v>4.763004773589489</v>
+        <v>0.01779337213885181</v>
       </c>
       <c r="S123" t="inlineStr">
         <is>
@@ -19685,17 +19685,17 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D184</t>
         </is>
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Accident caused by venomous animals</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>毒性动物伤害</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -19714,55 +19714,41 @@
         </is>
       </c>
       <c r="N124" t="n">
-        <v>1597</v>
+        <v>26801</v>
       </c>
       <c r="O124" t="n">
-        <v>1597</v>
+        <v>26801</v>
       </c>
       <c r="R124" t="n">
-        <v>0.7477898764670088</v>
+        <v>12.54947807087809</v>
       </c>
       <c r="S124" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U124" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA124" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO124" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP124" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ124" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS124" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR124" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS124" t="inlineStr"/>
       <c r="AT124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU124" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV124" t="inlineStr">
@@ -19829,7 +19815,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -19844,17 +19830,17 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D191</t>
         </is>
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Exogenous poisoning</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>外源性中毒</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -19873,130 +19859,41 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>1597</v>
+        <v>10172</v>
       </c>
       <c r="O125" t="n">
-        <v>1597</v>
-      </c>
-      <c r="U125" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="V125" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W125" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X125" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y125" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z125" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
-      <c r="AA125" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
-      <c r="AB125" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC125" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD125" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE125" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF125" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG125" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH125" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI125" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ125" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK125" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM125" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN125" t="b">
-        <v>1</v>
+        <v>10172</v>
+      </c>
+      <c r="R125" t="n">
+        <v>4.763004773589489</v>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
       </c>
       <c r="AO125" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP125" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ125" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS125" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR125" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS125" t="inlineStr"/>
       <c r="AT125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU125" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV125" t="inlineStr">
@@ -20078,70 +19975,84 @@
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>D021</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>登革热</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M126" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N126" t="n">
-        <v>28051</v>
+        <v>1597</v>
       </c>
       <c r="O126" t="n">
-        <v>28051</v>
+        <v>1597</v>
       </c>
       <c r="R126" t="n">
-        <v>13.13478636491926</v>
+        <v>0.7477898764670088</v>
       </c>
       <c r="S126" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA126" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
       <c r="AO126" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP126" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR126" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS126" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ126" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS126" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT126" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU126" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV126" t="inlineStr">
@@ -20208,7 +20119,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>public_projection</t>
+          <t>source_series_observation</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -20223,70 +20134,159 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D235</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N127" t="n">
-        <v>96</v>
+        <v>1597</v>
       </c>
       <c r="O127" t="n">
-        <v>96</v>
-      </c>
-      <c r="R127" t="n">
-        <v>0.04495167698236246</v>
-      </c>
-      <c r="S127" t="inlineStr">
-        <is>
-          <t>wpp_computed</t>
-        </is>
+        <v>1597</v>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W127" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA127" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB127" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC127" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD127" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE127" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF127" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG127" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH127" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI127" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ127" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK127" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM127" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN127" t="b">
+        <v>1</v>
       </c>
       <c r="AO127" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP127" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR127" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS127" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ127" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS127" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
       <c r="AT127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU127" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV127" t="inlineStr">
@@ -20368,17 +20368,17 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D021</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>登革热</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -20397,13 +20397,13 @@
         </is>
       </c>
       <c r="N128" t="n">
-        <v>4202</v>
+        <v>28051</v>
       </c>
       <c r="O128" t="n">
-        <v>4202</v>
+        <v>28051</v>
       </c>
       <c r="R128" t="n">
-        <v>1.967572361248823</v>
+        <v>13.13478636491926</v>
       </c>
       <c r="S128" t="inlineStr">
         <is>
@@ -20513,22 +20513,22 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -20542,13 +20542,13 @@
         </is>
       </c>
       <c r="N129" t="n">
-        <v>1</v>
+        <v>96</v>
       </c>
       <c r="O129" t="n">
-        <v>1</v>
+        <v>96</v>
       </c>
       <c r="R129" t="n">
-        <v>0.0004682466352329422</v>
+        <v>0.04495167698236246</v>
       </c>
       <c r="S129" t="inlineStr">
         <is>
@@ -20658,22 +20658,22 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L130" t="inlineStr">
@@ -20687,13 +20687,13 @@
         </is>
       </c>
       <c r="N130" t="n">
-        <v>1</v>
+        <v>4202</v>
       </c>
       <c r="O130" t="n">
-        <v>1</v>
+        <v>4202</v>
       </c>
       <c r="R130" t="n">
-        <v>0.0004682466352329422</v>
+        <v>1.967572361248823</v>
       </c>
       <c r="S130" t="inlineStr">
         <is>
@@ -20803,22 +20803,22 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -20832,13 +20832,13 @@
         </is>
       </c>
       <c r="N131" t="n">
-        <v>2970</v>
+        <v>1</v>
       </c>
       <c r="O131" t="n">
-        <v>2970</v>
+        <v>1</v>
       </c>
       <c r="R131" t="n">
-        <v>1.390692506641839</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S131" t="inlineStr">
         <is>
@@ -20948,17 +20948,17 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -20977,55 +20977,41 @@
         </is>
       </c>
       <c r="N132" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O132" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="R132" t="n">
-        <v>0.004682466352329423</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S132" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA132" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO132" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP132" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ132" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS132" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR132" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS132" t="inlineStr"/>
       <c r="AT132" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU132" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV132" t="inlineStr">
@@ -21092,212 +21078,516 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>D184</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Accident caused by venomous animals</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>毒性动物伤害</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N133" t="n">
+        <v>2970</v>
+      </c>
+      <c r="O133" t="n">
+        <v>2970</v>
+      </c>
+      <c r="R133" t="n">
+        <v>1.390692506641839</v>
+      </c>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO133" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP133" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR133" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS133" t="inlineStr"/>
+      <c r="AT133" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU133" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV133" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW133" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX133" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY133" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ133" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA133" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB133" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC133" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N134" t="n">
+        <v>10</v>
+      </c>
+      <c r="O134" t="n">
+        <v>10</v>
+      </c>
+      <c r="R134" t="n">
+        <v>0.004682466352329423</v>
+      </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AA134" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO134" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP134" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ134" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS134" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT134" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU134" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV134" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW134" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX134" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY134" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ134" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA134" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB134" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC134" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
           <t>source_series_observation</t>
         </is>
       </c>
-      <c r="F133" t="inlineStr">
+      <c r="F135" t="inlineStr">
         <is>
           <t>BR</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr">
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
         <is>
           <t>D235</t>
         </is>
       </c>
-      <c r="I133" t="inlineStr">
+      <c r="I135" t="inlineStr">
         <is>
           <t>Meningitis (all reported etiologies)</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr">
+      <c r="J135" t="inlineStr">
         <is>
           <t>脑膜炎（全部报告病因）</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr">
+      <c r="K135" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="L133" t="inlineStr">
+      <c r="L135" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr">
+      <c r="M135" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="N133" t="n">
+      <c r="N135" t="n">
         <v>10</v>
       </c>
-      <c r="O133" t="n">
+      <c r="O135" t="n">
         <v>10</v>
       </c>
-      <c r="U133" t="inlineStr">
+      <c r="U135" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="V133" t="inlineStr">
+      <c r="V135" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="W133" t="inlineStr">
+      <c r="W135" t="inlineStr">
         <is>
           <t>SRC_BR_SINAN</t>
         </is>
       </c>
-      <c r="X133" t="inlineStr">
+      <c r="X135" t="inlineStr">
         <is>
           <t>Meningitis</t>
         </is>
       </c>
-      <c r="Y133" t="inlineStr">
+      <c r="Y135" t="inlineStr">
         <is>
           <t>case_notifications</t>
         </is>
       </c>
-      <c r="Z133" t="inlineStr">
+      <c r="Z135" t="inlineStr">
         <is>
           <t>notification</t>
         </is>
       </c>
-      <c r="AA133" t="inlineStr">
+      <c r="AA135" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
       </c>
-      <c r="AB133" t="inlineStr">
+      <c r="AB135" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="AC133" t="inlineStr">
+      <c r="AC135" t="inlineStr">
         <is>
           <t>country:BR:national</t>
         </is>
       </c>
-      <c r="AD133" t="inlineStr">
+      <c r="AD135" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="AE133" t="inlineStr">
+      <c r="AE135" t="inlineStr">
         <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="AF133" t="inlineStr">
+      <c r="AF135" t="inlineStr">
         <is>
           <t>conditional</t>
         </is>
       </c>
-      <c r="AG133" t="inlineStr">
+      <c r="AG135" t="inlineStr">
         <is>
           <t>reported_aggregate</t>
         </is>
       </c>
-      <c r="AH133" t="inlineStr">
+      <c r="AH135" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="AI133" t="inlineStr">
+      <c r="AI135" t="inlineStr">
         <is>
           <t>missing_is_unknown</t>
         </is>
       </c>
-      <c r="AJ133" t="inlineStr">
+      <c r="AJ135" t="inlineStr">
         <is>
           <t>BR_SINAN_MENI_current</t>
         </is>
       </c>
-      <c r="AK133" t="inlineStr">
+      <c r="AK135" t="inlineStr">
         <is>
           <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
         </is>
       </c>
-      <c r="AM133" t="inlineStr">
+      <c r="AM135" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>
       </c>
-      <c r="AN133" t="b">
+      <c r="AN135" t="b">
         <v>1</v>
       </c>
-      <c r="AO133" t="inlineStr">
+      <c r="AO135" t="inlineStr">
         <is>
           <t>mixed</t>
         </is>
       </c>
-      <c r="AP133" t="inlineStr">
+      <c r="AP135" t="inlineStr">
         <is>
           <t>single_series</t>
         </is>
       </c>
-      <c r="AQ133" t="inlineStr">
+      <c r="AQ135" t="inlineStr">
         <is>
           <t>legacy_gap_fill</t>
         </is>
       </c>
-      <c r="AS133" t="inlineStr">
+      <c r="AS135" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="AT133" t="n">
+      <c r="AT135" t="n">
         <v>1</v>
       </c>
-      <c r="AU133" t="inlineStr">
+      <c r="AU135" t="inlineStr">
         <is>
           <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
-      <c r="AV133" t="inlineStr">
-        <is>
-          <t>sinan_datasus</t>
-        </is>
-      </c>
-      <c r="AW133" t="inlineStr">
-        <is>
-          <t>Brazil DATASUS SINAN</t>
-        </is>
-      </c>
-      <c r="AX133" t="inlineStr">
-        <is>
-          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
-        </is>
-      </c>
-      <c r="AY133" t="inlineStr">
-        <is>
-          <t>ftp_dbc</t>
-        </is>
-      </c>
-      <c r="AZ133" t="inlineStr">
-        <is>
-          <t>sinan_datasus</t>
-        </is>
-      </c>
-      <c r="BA133" t="inlineStr">
-        <is>
-          <t>Brazil DATASUS SINAN</t>
-        </is>
-      </c>
-      <c r="BB133" t="inlineStr">
-        <is>
-          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
-        </is>
-      </c>
-      <c r="BC133" t="inlineStr">
+      <c r="AV135" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW135" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX135" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY135" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ135" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA135" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB135" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC135" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -21419,7 +21709,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10">
@@ -21429,7 +21719,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11">
@@ -21481,7 +21771,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1091084</v>
+        <v>1091436</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-28 14:16:46 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -3078,7 +3078,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK33" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
@@ -11089,7 +11089,7 @@
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK69" t="inlineStr">
@@ -11328,7 +11328,7 @@
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK70" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK93" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK95" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK99" t="inlineStr">
@@ -16105,7 +16105,7 @@
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28</t>
+          <t>globalid-disease-ontology:2026.08.28.1</t>
         </is>
       </c>
       <c r="AK100" t="inlineStr">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-28 14:53:38 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -3078,7 +3078,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK33" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
@@ -11089,7 +11089,7 @@
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK69" t="inlineStr">
@@ -11328,7 +11328,7 @@
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK70" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK93" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK95" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK99" t="inlineStr">
@@ -16105,7 +16105,7 @@
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.1</t>
+          <t>globalid-disease-ontology:2026.08.28.2</t>
         </is>
       </c>
       <c r="AK100" t="inlineStr">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-30 02:27:24 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -3078,7 +3078,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="AJ33" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK33" t="inlineStr">
@@ -8056,7 +8056,7 @@
       </c>
       <c r="AJ49" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK49" t="inlineStr">
@@ -11089,7 +11089,7 @@
       </c>
       <c r="AJ69" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK69" t="inlineStr">
@@ -11328,7 +11328,7 @@
       </c>
       <c r="AJ70" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK70" t="inlineStr">
@@ -14785,7 +14785,7 @@
       </c>
       <c r="AJ93" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK93" t="inlineStr">
@@ -15178,7 +15178,7 @@
       </c>
       <c r="AJ95" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK95" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="AJ99" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK99" t="inlineStr">
@@ -16105,7 +16105,7 @@
       </c>
       <c r="AJ100" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.08.28.2</t>
+          <t>globalid-disease-ontology:2026.08.30.1</t>
         </is>
       </c>
       <c r="AK100" t="inlineStr">
@@ -16711,13 +16711,13 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="O104" t="n">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="R104" t="n">
-        <v>0.1755924882123533</v>
+        <v>0.1765289814828192</v>
       </c>
       <c r="S104" t="inlineStr">
         <is>
@@ -18554,13 +18554,13 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>219</v>
+        <v>297</v>
       </c>
       <c r="O116" t="n">
-        <v>219</v>
+        <v>297</v>
       </c>
       <c r="R116" t="n">
-        <v>0.1025460131160144</v>
+        <v>0.1390692506641839</v>
       </c>
       <c r="S116" t="inlineStr">
         <is>
@@ -19424,13 +19424,13 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="O122" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="R122" t="n">
-        <v>0.02294408512641417</v>
+        <v>0.03277726446630596</v>
       </c>
       <c r="S122" t="inlineStr">
         <is>
@@ -20513,22 +20513,22 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>D051</t>
+          <t>D028</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Zika virus disease</t>
+          <t>Pertussis</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>寨卡病毒病</t>
+          <t>百日咳</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Viral</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
@@ -20542,13 +20542,13 @@
         </is>
       </c>
       <c r="N129" t="n">
-        <v>96</v>
+        <v>41</v>
       </c>
       <c r="O129" t="n">
-        <v>96</v>
+        <v>41</v>
       </c>
       <c r="R129" t="n">
-        <v>0.04495167698236246</v>
+        <v>0.01919811204455063</v>
       </c>
       <c r="S129" t="inlineStr">
         <is>
@@ -20658,17 +20658,17 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>D052</t>
+          <t>D051</t>
         </is>
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Chikungunya</t>
+          <t>Zika virus disease</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>基孔肯雅热</t>
+          <t>寨卡病毒病</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -20687,13 +20687,13 @@
         </is>
       </c>
       <c r="N130" t="n">
-        <v>4202</v>
+        <v>96</v>
       </c>
       <c r="O130" t="n">
-        <v>4202</v>
+        <v>96</v>
       </c>
       <c r="R130" t="n">
-        <v>1.967572361248823</v>
+        <v>0.04495167698236246</v>
       </c>
       <c r="S130" t="inlineStr">
         <is>
@@ -20803,22 +20803,22 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>D120</t>
+          <t>D052</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Tetanus</t>
+          <t>Chikungunya</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>破伤风</t>
+          <t>基孔肯雅热</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Bacterial</t>
+          <t>Viral</t>
         </is>
       </c>
       <c r="L131" t="inlineStr">
@@ -20832,13 +20832,13 @@
         </is>
       </c>
       <c r="N131" t="n">
-        <v>1</v>
+        <v>4202</v>
       </c>
       <c r="O131" t="n">
-        <v>1</v>
+        <v>4202</v>
       </c>
       <c r="R131" t="n">
-        <v>0.0004682466352329422</v>
+        <v>1.967572361248823</v>
       </c>
       <c r="S131" t="inlineStr">
         <is>
@@ -20948,22 +20948,22 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>D178</t>
+          <t>D120</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Acute flaccid paralysis</t>
+          <t>Tetanus</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>急性无力肢体麻痹</t>
+          <t>破伤风</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Bacterial</t>
         </is>
       </c>
       <c r="L132" t="inlineStr">
@@ -20977,13 +20977,13 @@
         </is>
       </c>
       <c r="N132" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="O132" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="R132" t="n">
-        <v>0.0004682466352329422</v>
+        <v>0.004214219717096481</v>
       </c>
       <c r="S132" t="inlineStr">
         <is>
@@ -21093,17 +21093,17 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>D184</t>
+          <t>D178</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Accident caused by venomous animals</t>
+          <t>Acute flaccid paralysis</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>毒性动物伤害</t>
+          <t>急性无力肢体麻痹</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -21122,13 +21122,13 @@
         </is>
       </c>
       <c r="N133" t="n">
-        <v>2970</v>
+        <v>1</v>
       </c>
       <c r="O133" t="n">
-        <v>2970</v>
+        <v>1</v>
       </c>
       <c r="R133" t="n">
-        <v>1.390692506641839</v>
+        <v>0.0004682466352329422</v>
       </c>
       <c r="S133" t="inlineStr">
         <is>
@@ -21238,17 +21238,17 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>D235</t>
+          <t>D184</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Meningitis (all reported etiologies)</t>
+          <t>Accident caused by venomous animals</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>脑膜炎（全部报告病因）</t>
+          <t>毒性动物伤害</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -21267,55 +21267,41 @@
         </is>
       </c>
       <c r="N134" t="n">
-        <v>10</v>
+        <v>2970</v>
       </c>
       <c r="O134" t="n">
-        <v>10</v>
+        <v>2970</v>
       </c>
       <c r="R134" t="n">
-        <v>0.004682466352329423</v>
+        <v>1.390692506641839</v>
       </c>
       <c r="S134" t="inlineStr">
         <is>
           <t>wpp_computed</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="AA134" t="inlineStr">
-        <is>
-          <t>monthly</t>
-        </is>
-      </c>
       <c r="AO134" t="inlineStr">
         <is>
-          <t>mixed</t>
+          <t>legacy_fallback</t>
         </is>
       </c>
       <c r="AP134" t="inlineStr">
         <is>
-          <t>single_series</t>
-        </is>
-      </c>
-      <c r="AQ134" t="inlineStr">
-        <is>
-          <t>legacy_gap_fill</t>
-        </is>
-      </c>
-      <c r="AS134" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR134" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS134" t="inlineStr"/>
       <c r="AT134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU134" t="inlineStr">
         <is>
-          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
         </is>
       </c>
       <c r="AV134" t="inlineStr">
@@ -21382,7 +21368,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>source_series_observation</t>
+          <t>public_projection</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -21431,98 +21417,23 @@
       <c r="O135" t="n">
         <v>10</v>
       </c>
+      <c r="R135" t="n">
+        <v>0.004682466352329423</v>
+      </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
       <c r="U135" t="inlineStr">
         <is>
           <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
         </is>
       </c>
-      <c r="V135" t="inlineStr">
-        <is>
-          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
-        </is>
-      </c>
-      <c r="W135" t="inlineStr">
-        <is>
-          <t>SRC_BR_SINAN</t>
-        </is>
-      </c>
-      <c r="X135" t="inlineStr">
-        <is>
-          <t>Meningitis</t>
-        </is>
-      </c>
-      <c r="Y135" t="inlineStr">
-        <is>
-          <t>case_notifications</t>
-        </is>
-      </c>
-      <c r="Z135" t="inlineStr">
-        <is>
-          <t>notification</t>
-        </is>
-      </c>
       <c r="AA135" t="inlineStr">
         <is>
           <t>monthly</t>
         </is>
-      </c>
-      <c r="AB135" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="AC135" t="inlineStr">
-        <is>
-          <t>country:BR:national</t>
-        </is>
-      </c>
-      <c r="AD135" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="AE135" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="AF135" t="inlineStr">
-        <is>
-          <t>conditional</t>
-        </is>
-      </c>
-      <c r="AG135" t="inlineStr">
-        <is>
-          <t>reported_aggregate</t>
-        </is>
-      </c>
-      <c r="AH135" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="AI135" t="inlineStr">
-        <is>
-          <t>missing_is_unknown</t>
-        </is>
-      </c>
-      <c r="AJ135" t="inlineStr">
-        <is>
-          <t>BR_SINAN_MENI_current</t>
-        </is>
-      </c>
-      <c r="AK135" t="inlineStr">
-        <is>
-          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
-        </is>
-      </c>
-      <c r="AM135" t="inlineStr">
-        <is>
-          <t>provisional</t>
-        </is>
-      </c>
-      <c r="AN135" t="b">
-        <v>1</v>
       </c>
       <c r="AO135" t="inlineStr">
         <is>
@@ -21588,6 +21499,240 @@
         </is>
       </c>
       <c r="BC135" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>br</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>D235</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Meningitis (all reported etiologies)</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>脑膜炎（全部报告病因）</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N136" t="n">
+        <v>10</v>
+      </c>
+      <c r="O136" t="n">
+        <v>10</v>
+      </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="V136" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="W136" t="inlineStr">
+        <is>
+          <t>SRC_BR_SINAN</t>
+        </is>
+      </c>
+      <c r="X136" t="inlineStr">
+        <is>
+          <t>Meningitis</t>
+        </is>
+      </c>
+      <c r="Y136" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z136" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA136" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB136" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC136" t="inlineStr">
+        <is>
+          <t>country:BR:national</t>
+        </is>
+      </c>
+      <c r="AD136" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE136" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF136" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG136" t="inlineStr">
+        <is>
+          <t>reported_aggregate</t>
+        </is>
+      </c>
+      <c r="AH136" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI136" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ136" t="inlineStr">
+        <is>
+          <t>BR_SINAN_MENI_current</t>
+        </is>
+      </c>
+      <c r="AK136" t="inlineStr">
+        <is>
+          <t>Brazil SINAN MENI file family spans reported meningitis etiologies and must not be interpreted as bacterial meningitis only.</t>
+        </is>
+      </c>
+      <c r="AM136" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+      <c r="AN136" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO136" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="AP136" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ136" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS136" t="inlineStr">
+        <is>
+          <t>SER_BR_MENINGITIS_ALL_ETIOLOGIES_MENI</t>
+        </is>
+      </c>
+      <c r="AT136" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU136" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
+        </is>
+      </c>
+      <c r="AV136" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="AW136" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="AX136" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="AY136" t="inlineStr">
+        <is>
+          <t>ftp_dbc</t>
+        </is>
+      </c>
+      <c r="AZ136" t="inlineStr">
+        <is>
+          <t>sinan_datasus</t>
+        </is>
+      </c>
+      <c r="BA136" t="inlineStr">
+        <is>
+          <t>Brazil DATASUS SINAN</t>
+        </is>
+      </c>
+      <c r="BB136" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
+      <c r="BC136" t="inlineStr">
         <is>
           <t>ftp_dbc</t>
         </is>
@@ -21709,7 +21854,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10">
@@ -21719,7 +21864,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11">
@@ -21771,7 +21916,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1091436</v>
+        <v>1091586</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-04 02:12:38 UTC
</commit_message>
<xml_diff>
--- a/countries/br/2026-2029.xlsx
+++ b/countries/br/2026-2029.xlsx
@@ -18409,13 +18409,13 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>44692</v>
+        <v>42567</v>
       </c>
       <c r="O115" t="n">
-        <v>44692</v>
+        <v>42567</v>
       </c>
       <c r="R115" t="n">
-        <v>20.92687862183066</v>
+        <v>19.93185452196065</v>
       </c>
       <c r="S115" t="inlineStr">
         <is>
@@ -18989,13 +18989,13 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>1169</v>
+        <v>1258</v>
       </c>
       <c r="O119" t="n">
-        <v>1169</v>
+        <v>1258</v>
       </c>
       <c r="R119" t="n">
-        <v>0.5473803165873095</v>
+        <v>0.5890542671230413</v>
       </c>
       <c r="S119" t="inlineStr">
         <is>
@@ -19134,13 +19134,13 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>10988</v>
+        <v>11345</v>
       </c>
       <c r="O120" t="n">
-        <v>10988</v>
+        <v>11345</v>
       </c>
       <c r="R120" t="n">
-        <v>5.14509402793957</v>
+        <v>5.31225807671773</v>
       </c>
       <c r="S120" t="inlineStr">
         <is>
@@ -20397,13 +20397,13 @@
         </is>
       </c>
       <c r="N128" t="n">
-        <v>28051</v>
+        <v>37468</v>
       </c>
       <c r="O128" t="n">
-        <v>28051</v>
+        <v>37468</v>
       </c>
       <c r="R128" t="n">
-        <v>13.13478636491926</v>
+        <v>17.54426492890788</v>
       </c>
       <c r="S128" t="inlineStr">
         <is>
@@ -20687,13 +20687,13 @@
         </is>
       </c>
       <c r="N130" t="n">
-        <v>96</v>
+        <v>244</v>
       </c>
       <c r="O130" t="n">
-        <v>96</v>
+        <v>244</v>
       </c>
       <c r="R130" t="n">
-        <v>0.04495167698236246</v>
+        <v>0.1142521789968379</v>
       </c>
       <c r="S130" t="inlineStr">
         <is>
@@ -20832,13 +20832,13 @@
         </is>
       </c>
       <c r="N131" t="n">
-        <v>4202</v>
+        <v>6520</v>
       </c>
       <c r="O131" t="n">
-        <v>4202</v>
+        <v>6520</v>
       </c>
       <c r="R131" t="n">
-        <v>1.967572361248823</v>
+        <v>3.052968061718784</v>
       </c>
       <c r="S131" t="inlineStr">
         <is>
@@ -21916,7 +21916,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1091586</v>
+        <v>1101790</v>
       </c>
     </row>
     <row r="16">

</xml_diff>